<commit_message>
chore: update address tested
</commit_message>
<xml_diff>
--- a/instatus-tested-addresses/instatus-addresses.xlsx
+++ b/instatus-tested-addresses/instatus-addresses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">Addresses</t>
   </si>
@@ -158,9 +158,6 @@
   </si>
   <si>
     <t xml:space="preserve">32 Rue Robert Desnos, 34070 Montpellier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 Bisserweg, 1238 Grund Luxembourg</t>
   </si>
 </sst>
 </file>
@@ -170,7 +167,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -199,12 +196,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="3">
@@ -255,20 +246,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -464,243 +459,241 @@
   <dimension ref="A1:A1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="99.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="99.75"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="3" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="3" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+      <c r="A46" s="1" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>46</v>
-      </c>
+      <c r="A47" s="4"/>
     </row>
     <row r="48" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>